<commit_message>
Tracker: S3 and P1 back to DONE after local restore
Both deliverables are in the tree again, so the sheet says so. Adds a Work Log
row recording the revert-then-restore round trip and why the restore was done
at file level rather than by reverting the revert.

Local only — not pushed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013waY6TGwwKkqWdtdpdiQ7V
</commit_message>
<xml_diff>
--- a/Shagun_Task_Tracker.xlsx
+++ b/Shagun_Task_Tracker.xlsx
@@ -66,7 +66,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4DFEC"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -579,7 +579,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="92" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>S3</t>
@@ -602,7 +602,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Reverted</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -610,7 +610,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Built IntentScenarioComposer with one scripted tree per mandated intent — depth varied by structural distinctness (single-turn lookup, multi-turn slot filling, out-of-scope refusal, ambiguity-&gt;clarify, and CV-17 mid-conversation requirement change as a real branching tree). Shipped BOTH halves of the §16.6 Phase-2 seam: ReplySource protocol (ScriptedReplySource for Phase 1) and Evaluator protocol (ExactExpectationEvaluator, judges a transcript not the script so it survives LLM-generated replies). All claims grounded in the same World the booking-API mock reads. Split delivered_excludes (claim WRONG vs live data, must never be delivered) from superseded_tokens (claim CORRECT when said, then obsoleted — must not reach the final confirmation); conflating them made one of the two cases silently stop testing anything.</t>
@@ -618,7 +622,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>REVERTED 2026-09-01 — work is not in the tree. Fully recoverable: git revert --no-commit &lt;revert-sha&gt;  (or cherry-pick 9840cb0, 78aedf0). Was: generator/intents.py, models.py, pipeline.py, cli.py, tests/test_conversation_intents.py — 73 tests green.</t>
+          <t>generator/intents.py (new), models.py, pipeline.py, cli.py, tests/test_conversation_intents.py — 73 tests green. Reverted then restored 2026-09-01; in the tree and green. Local only, not pushed.</t>
         </is>
       </c>
     </row>
@@ -917,7 +921,7 @@
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
     </row>
-    <row r="15" ht="34" customHeight="1">
+    <row r="15" ht="92" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>P1</t>
@@ -940,7 +944,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Reverted</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -948,7 +952,11 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Wrote POA/18: split the module dependency graph into two tracks so no module gets built twice, mapped cross-track contract points, and defined the daily push/merge routine. Corrected an early error in it — B1 does NOT block Prasad's A5/A6/A8, because the M13 contract already exists. Confirmed track ownership after Prasad accepted Track A.</t>
@@ -956,7 +964,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>REVERTED 2026-09-01 — POA/18 is not in the tree. Recoverable from d1f6987, 3f444b8.</t>
+          <t>POA/18_Team_Work_Split_and_Git_Workflow.md + POA/00 index row. Reverted then restored 2026-09-01; in the tree. Local only, not pushed.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1232,6 +1240,33 @@
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>local only</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>S3 / P1</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Restored both reverted deliverables locally at Shagun's request — S3 first, then POA/18. Restored at file level from 78aedf0 / b54edb8 rather than by reverting the revert, so each came back independently and history stays readable. Restoring POA/18 also re-validated the 'see POA/18 §4' pointer in generator/models.py, which was dangling in between.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Working tree == b54edb8 (plus tracker improvements); 73 tests green</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>local only</t>
         </is>

</xml_diff>